<commit_message>
fix remaining extraction accuracy issues in hybrid_procurement_extractor
</commit_message>
<xml_diff>
--- a/output/output.xlsx
+++ b/output/output.xlsx
@@ -3097,7 +3097,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -3106,11 +3106,7 @@
           <t>01</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>SEMÁFORO LED DE TRÁFICO 1 X 12 in DE POLICARBONATO</t>
-        </is>
-      </c>
+      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
@@ -3138,30 +3134,22 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
+          <t>SEMÁFORO LED DE TRÁFICO 1 X 12 in DE POLICARBONATO  Nombre comercial: Óptico para semáforo ciclista.  Año de fabricación: Mínimo 2022  Emitirá 02 señales: Rojo Estático y Verde Dinámico.  Diámetro nominal de la unidad óptica 300 mm  IMPORTANTE: El óptico para semáforo ciclista 300 mm, debe cumplir con las Características Específicas descritas en el numeral 3.2.1.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SEMÁFORO LED DE TRÁFICO 1 X 12 in DE POLICARBONATO  Nombre comercial: Óptico para semáforo ciclista.  Año de fabricación: Mínimo 2022  Emitirá 02 señales: Rojo Estático y Verde Dinámico.  Diámetro nominal de la unidad óptica 300 mm  IMPORTANTE: El óptico para semáforo ciclista 300 mm, debe cumplir con las Características Específicas descritas en el numeral 3.2.1.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
           <t>01</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
@@ -3667,16 +3655,8 @@
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios a contratar se encuentran en el listado de bienes y servicios comunes de la Subasta Inversa Electrónica</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios a contratar se encuentran en el listado de bienes y servicios comunes de la Subasta Inversa Electrónica</t>
-        </is>
-      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
@@ -3714,16 +3694,8 @@
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios se encuentran en algún catálogo del Acuerdo Marco</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios se encuentran en algún catálogo del Acuerdo Marco</t>
-        </is>
-      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
@@ -3761,16 +3733,8 @@
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios se encuentran en las fichas de homologación</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Los bienes o servicios se encuentran en las fichas de homologación</t>
-        </is>
-      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
@@ -3808,16 +3772,8 @@
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>13. RESOLUCIÓN DE CONTRATO U O/C</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>13. RESOLUCIÓN DE CONTRATO U O/C</t>
-        </is>
-      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>

</xml_diff>